<commit_message>
scan: seg7 2026-08-10 15:53 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-10.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-10.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O73"/>
+  <dimension ref="A1:O85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1481,21 +1481,21 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>7772</v>
+        <v>8043</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>耀穎</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>420.3488446535803</v>
+        <v>431.5052089023578</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>93.5</v>
+        <v>134.5</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,16 +1506,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>39.68948361826616</v>
+        <v>44.14716118827981</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>28.93126156662644</v>
+        <v>24.02946079670646</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.546429196405302</v>
+        <v>0.535550014133778</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2.152551939964338</v>
+        <v>0.627681496639255</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, foreign_buy_3d, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>8021</v>
+        <v>7772</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>尖點</t>
+          <t>耀穎</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>418.3155882950135</v>
+        <v>420.3488446535803</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>434.5</v>
+        <v>93.5</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>52.05529013866558</v>
+        <v>39.68948361826616</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>20.69803572716395</v>
+        <v>28.93126156662644</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1.174403439739875</v>
+        <v>0.546429196405302</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>9.231645425792481</v>
+        <v>2.152551939964338</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, foreign_buy_3d, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>8016</v>
+        <v>8021</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>矽創</t>
+          <t>尖點</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>411.5235967366355</v>
+        <v>418.3155882950135</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>311</v>
+        <v>434.5</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>56.46378831138386</v>
+        <v>52.05529013866558</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>17.96337136799711</v>
+        <v>20.69803572716395</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.8646728840768798</v>
+        <v>1.174403439739875</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>3.792988789761944</v>
+        <v>9.231645425792481</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>8028</v>
+        <v>8016</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>昇陽半導體</t>
+          <t>矽創</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>402.6669599431088</v>
+        <v>411.5235967366355</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>264</v>
+        <v>311</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,13 +1665,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>44.54530422854908</v>
+        <v>56.46378831138386</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>17.57807619073095</v>
+        <v>17.96337136799711</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.6245577589817797</v>
+        <v>0.8646728840768798</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-1.708332335542504</v>
+        <v>3.792988789761944</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6840</v>
+        <v>6902</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>GOGOLOOK</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>392.8704967562953</v>
+        <v>406.2551900768641</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>66</v>
+        <v>127.5</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>57.82766936495749</v>
+        <v>53.85628271342131</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>16.06491463565078</v>
+        <v>17.64518565979985</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.9263291014220169</v>
+        <v>1.510763084538744</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.9514661205781592</v>
+        <v>0.851508709826875</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>7730</v>
+        <v>8028</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>昇陽半導體</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>387.6791268571542</v>
+        <v>402.6669599431088</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>156</v>
+        <v>264</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>43.20025111397574</v>
+        <v>44.54530422854908</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>26.36568612964308</v>
+        <v>17.57807619073095</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.7395270184432883</v>
+        <v>0.6245577589817797</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.642135619025777</v>
+        <v>-1.708332335542504</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>7715</v>
+        <v>6840</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>裕山</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>374.4277684574971</v>
+        <v>392.8704967562953</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>33.7</v>
+        <v>66</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.5028733099393</v>
+        <v>57.82766936495749</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.74679255494288</v>
+        <v>16.06491463565078</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.8013024234762182</v>
+        <v>0.9263291014220169</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.2700211412288262</v>
+        <v>0.9514661205781592</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>7822</v>
+        <v>7722</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>倍利科</t>
+          <t>LINEPAY</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>365.2323470495224</v>
+        <v>390.2101336695713</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>873</v>
+        <v>293.5</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>46.30823784707533</v>
+        <v>50.67530614558645</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>23.81656058380574</v>
+        <v>22.59554852826844</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.7918153061430665</v>
+        <v>2.353905779174727</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>14.93350937883291</v>
+        <v>1.270975661211557</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6996</v>
+        <v>7730</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>355.8921281454355</v>
+        <v>387.6791268571542</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>178</v>
+        <v>156</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>47.66591625659076</v>
+        <v>43.20025111397574</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>19.49961166517138</v>
+        <v>26.36568612964308</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>2.110489189766993</v>
+        <v>0.7395270184432883</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.647444506647588</v>
+        <v>0.642135619025777</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>7788</v>
+        <v>6861</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>松川精密</t>
+          <t>睿生光電</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>352.5195590835073</v>
+        <v>376.064870366769</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>234.5</v>
+        <v>220.5</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>54.98764852813682</v>
+        <v>44.47111918058776</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>22.12007366637414</v>
+        <v>29.43897930262679</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1.318955949184313</v>
+        <v>1.410224858519075</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3.360942142263006</v>
+        <v>6.417485868615618</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>7820</v>
+        <v>7715</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>立盈</t>
+          <t>裕山</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>351.8418134944964</v>
+        <v>374.4277684574971</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>121</v>
+        <v>33.7</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>63.30789963826737</v>
+        <v>51.5028733099393</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>20.35642106830964</v>
+        <v>23.74679255494288</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.9907472841717752</v>
+        <v>0.8013024234762182</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.79172910875751</v>
+        <v>0.2700211412288262</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, adx_trending, cci_momentum</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6944</v>
+        <v>8040</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>兆聯實業</t>
+          <t>九暘</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>351.0755103214687</v>
+        <v>368.8111411392525</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>755</v>
+        <v>76</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>39.45251522109933</v>
+        <v>46.85589731329837</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.1721825855067</v>
+        <v>25.85907546799718</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.7053780360589114</v>
+        <v>0.9100083479036618</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.6187859460429763</v>
+        <v>1.377558288232594</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6916</v>
+        <v>8042</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>金山電</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>345.518600701358</v>
+        <v>367.5068505064758</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18.85</v>
+        <v>114</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>48.90059320173452</v>
+        <v>42.98922321051411</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>14.2771055660218</v>
+        <v>26.66754042625202</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.7998603975060667</v>
+        <v>1.4602350073193</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.0135482809874605</v>
+        <v>1.558382140541465</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>7631</v>
+        <v>7822</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>聚賢研發-創</t>
+          <t>倍利科</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>343.2182848273715</v>
+        <v>365.2323470495224</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>138.5</v>
+        <v>873</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>51.17164742818062</v>
+        <v>46.30823784707533</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>10.58711842514319</v>
+        <v>23.81656058380574</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.890638086684824</v>
+        <v>0.7918153061430665</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.2622101797018885</v>
+        <v>14.93350937883291</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6903</v>
+        <v>6996</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>巨漢</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>341.4428762712377</v>
+        <v>355.8921281454355</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>315</v>
+        <v>178</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>41.47879025893688</v>
+        <v>47.66591625659076</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>23.36529971780059</v>
+        <v>19.49961166517138</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.8947602208992691</v>
+        <v>2.110489189766993</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.5765925389202131</v>
+        <v>1.647444506647588</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>7556</v>
+        <v>7788</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>意德士</t>
+          <t>松川精密</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>341.1909086197857</v>
+        <v>352.5195590835073</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>223</v>
+        <v>234.5</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>44.06656304659347</v>
+        <v>54.98764852813682</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>33.57384172151545</v>
+        <v>22.12007366637414</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.4930129006142312</v>
+        <v>1.318955949184313</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>3.139613451160402</v>
+        <v>3.360942142263006</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6962</v>
+        <v>7820</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>奕力-KY</t>
+          <t>立盈</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>340.1052401015757</v>
+        <v>351.8418134944964</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>34.15</v>
+        <v>121</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>54.43930160255238</v>
+        <v>63.30789963826737</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>26.47641270677479</v>
+        <v>20.35642106830964</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>2.337111937942113</v>
+        <v>0.9907472841717752</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.3074808686727293</v>
+        <v>1.79172910875751</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, adx_trending, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6947</v>
+        <v>6944</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>兆聯實業</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>333.6386631497986</v>
+        <v>351.0755103214687</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>78.40000000000001</v>
+        <v>755</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>48.11603220260852</v>
+        <v>39.45251522109933</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20.00408778315144</v>
+        <v>24.1721825855067</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.3776519107627281</v>
+        <v>0.7053780360589114</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.9533044677711456</v>
+        <v>-0.6187859460429763</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>7769</v>
+        <v>6916</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>鴻勁</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>333.3384933418082</v>
+        <v>345.518600701358</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>6280</v>
+        <v>18.85</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>49.21114938393828</v>
+        <v>48.90059320173452</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>11.96144274988899</v>
+        <v>14.2771055660218</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.9154755827488124</v>
+        <v>0.7998603975060667</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>60.8953777667781</v>
+        <v>0.0135482809874605</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>8011</v>
+        <v>7631</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>台通</t>
+          <t>聚賢研發-創</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>332.3622190746955</v>
+        <v>343.2182848273715</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>16.5</v>
+        <v>138.5</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>46.82237955311683</v>
+        <v>51.17164742818062</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>27.93650649771128</v>
+        <v>10.58711842514319</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.3623876736930858</v>
+        <v>1.890638086684824</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0877836687983575</v>
+        <v>-0.2622101797018885</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6951</v>
+        <v>6903</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>巨漢</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>331.9613606219231</v>
+        <v>341.4428762712377</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>71.40000000000001</v>
+        <v>315</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>38.06197508141646</v>
+        <v>41.47879025893688</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>38.31744810274584</v>
+        <v>23.36529971780059</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1.36819847716718</v>
+        <v>0.8947602208992691</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.2185891576503196</v>
+        <v>0.5765925389202131</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>7792</v>
+        <v>7556</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>安葆</t>
+          <t>意德士</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>319.3551689189641</v>
+        <v>341.1909086197857</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>214.5</v>
+        <v>223</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>47.77540112805456</v>
+        <v>44.06656304659347</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>31.02575142393854</v>
+        <v>33.57384172151545</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.8361148088159112</v>
+        <v>0.4930129006142312</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>1</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>3.431447458833473</v>
+        <v>3.139613451160402</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>7712</v>
+        <v>6962</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>博盛半導體</t>
+          <t>奕力-KY</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>279.3662481200215</v>
+        <v>340.1052401015757</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>148</v>
+        <v>34.15</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>49.44297980530506</v>
+        <v>54.43930160255238</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>24.40210027731012</v>
+        <v>26.47641270677479</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1.003335673483302</v>
+        <v>2.337111937942113</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>1.999544596433511</v>
+        <v>0.3074808686727293</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>7818</v>
+        <v>6947</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>278.8178727364322</v>
+        <v>333.6386631497986</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>63</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>35.60140950276744</v>
+        <v>48.11603220260852</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>34.42993761010147</v>
+        <v>20.00408778315144</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1.334145359594396</v>
+        <v>0.3776519107627281</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.4636830399100147</v>
+        <v>0.9533044677711456</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6971</v>
+        <v>7769</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>鴻勁</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>261.7270042559304</v>
+        <v>333.3384933418082</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>25.6</v>
+        <v>6280</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>33.91237872203467</v>
+        <v>49.21114938393828</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>17.01885669953462</v>
+        <v>11.96144274988899</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.8672591330968397</v>
+        <v>0.9154755827488124</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.0832816962732336</v>
+        <v>60.8953777667781</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6994</v>
+        <v>8011</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>台通</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>261.4068056261588</v>
+        <v>332.3622190746955</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>36.95</v>
+        <v>16.5</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>32.83487720384579</v>
+        <v>46.82237955311683</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>37.20335097067832</v>
+        <v>27.93650649771128</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.039352681445436</v>
+        <v>0.3623876736930858</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.2860591208910428</v>
+        <v>0.0877836687983575</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6895</v>
+        <v>6951</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>259.0606006390066</v>
+        <v>331.9613606219231</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>118.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>38.55842070116779</v>
+        <v>38.06197508141646</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>26.65253592694184</v>
+        <v>38.31744810274584</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.707150545535427</v>
+        <v>1.36819847716718</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>1.010515000537925</v>
+        <v>0.2185891576503196</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2912,21 +2912,21 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6921</v>
+        <v>7792</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>安葆</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>258.3491585906293</v>
+        <v>319.3551689189641</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>65.2</v>
+        <v>214.5</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.70936219945977</v>
+        <v>47.77540112805456</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>27.28507203244613</v>
+        <v>31.02575142393854</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1.167351073303999</v>
+        <v>0.8361148088159112</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.7173881703814038</v>
+        <v>3.431447458833473</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2965,21 +2965,21 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6859</v>
+        <v>7721</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>253.8726662502864</v>
+        <v>303.7277100092821</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>99.7</v>
+        <v>62.9</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>36.50236058509879</v>
+        <v>46.96959264934583</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>28.1473739515334</v>
+        <v>25.42277511086672</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.385620120895477</v>
+        <v>0.2936804443314063</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.9242135344558536</v>
+        <v>0.6996548094949717</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6869</v>
+        <v>7712</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>博盛半導體</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>242.6743828855074</v>
+        <v>279.3662481200215</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>70.2</v>
+        <v>148</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>52.92645220861025</v>
+        <v>49.44297980530506</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>19.20256061100446</v>
+        <v>24.40210027731012</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1.084395523378353</v>
+        <v>1.003335673483302</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.7016466010087159</v>
+        <v>1.999544596433511</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>7768</v>
+        <v>7818</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>239.9041356068924</v>
+        <v>278.8178727364322</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>261.5</v>
+        <v>63</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>35.83878580896345</v>
+        <v>35.60140950276744</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>45.16833733265</v>
+        <v>34.42993761010147</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.4331677512119838</v>
+        <v>1.334145359594396</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>1.886270425394073</v>
+        <v>-0.4636830399100147</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6908</v>
+        <v>6971</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>239.5553009001952</v>
+        <v>261.7270042559304</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>32.9</v>
+        <v>25.6</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>36.12329248450961</v>
+        <v>33.91237872203467</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>31.5423807528287</v>
+        <v>17.01885669953462</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1.02796052631579</v>
+        <v>0.8672591330968397</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.07725547166748289</v>
+        <v>-0.0832816962732336</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6887</v>
+        <v>6994</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>236.8265361674669</v>
+        <v>261.4068056261588</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>36.05</v>
+        <v>36.95</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>47.83771172224126</v>
+        <v>32.83487720384579</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>17.00962407669346</v>
+        <v>37.20335097067832</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.2060087555679954</v>
+        <v>1.039352681445436</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.185212618965927</v>
+        <v>0.2860591208910428</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>7749</v>
+        <v>6895</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>230.2345308208552</v>
+        <v>259.0606006390066</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>355.5</v>
+        <v>118.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>44.64577207325237</v>
+        <v>38.55842070116779</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>32.27720967521438</v>
+        <v>26.65253592694184</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.6268777173692717</v>
+        <v>0.707150545535427</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>5.34143688898196</v>
+        <v>1.010515000537925</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6899</v>
+        <v>6921</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>224.3041518260263</v>
+        <v>258.3491585906293</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>50.7</v>
+        <v>65.2</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>38.06729527396745</v>
+        <v>51.70936219945977</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>23.54492871355304</v>
+        <v>27.28507203244613</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.4908126190059958</v>
+        <v>1.167351073303999</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.3486261016285426</v>
+        <v>0.7173881703814038</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6953</v>
+        <v>6859</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>220.6802644635352</v>
+        <v>253.8726662502864</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>223</v>
+        <v>99.7</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.95213263675682</v>
+        <v>36.50236058509879</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>9.894791767196232</v>
+        <v>28.1473739515334</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.3082033120190888</v>
+        <v>0.385620120895477</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>1.788417789291647</v>
+        <v>0.9242135344558536</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6873</v>
+        <v>6869</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>215.0974662222889</v>
+        <v>242.6743828855074</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>79</v>
+        <v>70.2</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.20207975417044</v>
+        <v>52.92645220861025</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.63486014762306</v>
+        <v>19.20256061100446</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.10646005076004</v>
+        <v>1.084395523378353</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.3468792592392931</v>
+        <v>0.7016466010087159</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6894</v>
+        <v>7768</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>209.6960034481655</v>
+        <v>239.9041356068924</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>346.5</v>
+        <v>261.5</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>53.05600793743652</v>
+        <v>35.83878580896345</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>16.31462079186515</v>
+        <v>45.16833733265</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.7580949872617595</v>
+        <v>0.4331677512119838</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>4.406072900351855</v>
+        <v>1.886270425394073</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6877</v>
+        <v>6908</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>209.4432275446592</v>
+        <v>239.5553009001952</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>127.5</v>
+        <v>32.9</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>52.24148104051165</v>
+        <v>36.12329248450961</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>18.53708461897214</v>
+        <v>31.5423807528287</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.8661062567621975</v>
+        <v>1.02796052631579</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>1.500200763685784</v>
+        <v>-0.07725547166748289</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>7402</v>
+        <v>6887</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>207.5863099348092</v>
+        <v>236.8265361674669</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>103</v>
+        <v>36.05</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>44.19251715783129</v>
+        <v>47.83771172224126</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.63468970003154</v>
+        <v>17.00962407669346</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.149618364569397</v>
+        <v>0.2060087555679954</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.7599105654133251</v>
+        <v>-0.185212618965927</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>7842</v>
+        <v>6906</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>204.0135455639476</v>
+        <v>233.0092844365423</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>91.59999999999999</v>
+        <v>71</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>53.00345780940963</v>
+        <v>40.56464498373511</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>10.26079279614132</v>
+        <v>29.34192093776815</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.6562574970012</v>
+        <v>0.9136662795199382</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>1.205609064200336</v>
+        <v>0.7920186934425986</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6967</v>
+        <v>7749</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>196.6235767539877</v>
+        <v>230.2345308208552</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>69.3</v>
+        <v>355.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,16 +3679,16 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>45.52480241209469</v>
+        <v>44.64577207325237</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>16.49585506093718</v>
+        <v>32.27720967521438</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.08774113964356781</v>
+        <v>0.6268777173692717</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.3162031130703682</v>
+        <v>5.34143688898196</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6924</v>
+        <v>6899</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>193.2275993596958</v>
+        <v>224.3041518260263</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>109</v>
+        <v>50.7</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>47.51677580480385</v>
+        <v>38.06729527396745</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.47828919063415</v>
+        <v>23.54492871355304</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.9272853552686484</v>
+        <v>0.4908126190059958</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>1.701399838645164</v>
+        <v>0.3486261016285426</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6854</v>
+        <v>6953</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>193.0424662116648</v>
+        <v>220.6802644635352</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>94.2</v>
+        <v>223</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>37.26115285406406</v>
+        <v>52.95213263675682</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>39.63792182044081</v>
+        <v>9.894791767196232</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.504827075497997</v>
+        <v>0.3082033120190888</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>1.504382211881563</v>
+        <v>1.788417789291647</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>7689</v>
+        <v>6873</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>180.6674511561264</v>
+        <v>215.0974662222889</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>171.5</v>
+        <v>79</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>28.20380236778568</v>
+        <v>43.20207975417044</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>32.172995789672</v>
+        <v>16.63486014762306</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.140115856278475</v>
+        <v>1.10646005076004</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-1.182610235517359</v>
+        <v>-0.3468792592392931</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6909</v>
+        <v>8034</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>170.0951339405282</v>
+        <v>214.1047081881592</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>41.85</v>
+        <v>19.1</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,16 +3891,16 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>42.40015852246751</v>
+        <v>39.79083766211048</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>30.11710488316989</v>
+        <v>36.10566422157577</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.6574252603047193</v>
+        <v>0.6850546000333173</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L65" s="2" t="n">
         <v>0</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.3705297194905128</v>
+        <v>0.1409505553634835</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3919,21 +3919,21 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>7703</v>
+        <v>6894</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>153.3959725847375</v>
+        <v>209.6960034481655</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>185</v>
+        <v>346.5</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>52.2358435862429</v>
+        <v>53.05600793743652</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>20.68008864281432</v>
+        <v>16.31462079186515</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.4279785520285751</v>
+        <v>0.7580949872617595</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>2.023106993773102</v>
+        <v>4.406072900351855</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>7770</v>
+        <v>8024</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>142.2583098809928</v>
+        <v>209.6240690164325</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>39.75</v>
+        <v>14.1</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>52.28709347745657</v>
+        <v>44.03815138841021</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>12.82793555296719</v>
+        <v>18.49613831537289</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.08076032497761131</v>
+        <v>0.6706454070423011</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.5688200717833749</v>
+        <v>-0.1398571671965818</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>7728</v>
+        <v>6877</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>126.305852728335</v>
+        <v>209.4432275446592</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>608</v>
+        <v>127.5</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>47.36484555352385</v>
+        <v>52.24148104051165</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>17.82074134149556</v>
+        <v>18.53708461897214</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.4318038724417933</v>
+        <v>0.8661062567621975</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>5.782353699127107</v>
+        <v>1.500200763685784</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6923</v>
+        <v>7402</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>125.6502179615506</v>
+        <v>207.5863099348092</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>76.7</v>
+        <v>103</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>50.55926572210412</v>
+        <v>44.19251715783129</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>10.95229127344426</v>
+        <v>20.63468970003154</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.6754157054475967</v>
+        <v>0.149618364569397</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.0820209368688771</v>
+        <v>-0.7599105654133251</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>7753</v>
+        <v>7842</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>124.1688204529087</v>
+        <v>204.0135455639476</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>37.85</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>41.6224675178943</v>
+        <v>53.00345780940963</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>13.06905315791652</v>
+        <v>10.26079279614132</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.3407396361467342</v>
+        <v>1.6562574970012</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0566640056100098</v>
+        <v>1.205609064200336</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6862</v>
+        <v>6967</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>114.7208036103052</v>
+        <v>196.6235767539877</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>149</v>
+        <v>69.3</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>47.30722977554326</v>
+        <v>45.52480241209469</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>22.42855587726057</v>
+        <v>16.49585506093718</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.475159423827381</v>
+        <v>0.08774113964356781</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>2.959759627101038</v>
+        <v>-0.3162031130703682</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>7810</v>
+        <v>6924</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>89.19630396848171</v>
+        <v>193.2275993596958</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>196</v>
+        <v>109</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>50.99644358545656</v>
+        <v>47.51677580480385</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14.912466551393</v>
+        <v>18.47828919063415</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.676627564028675</v>
+        <v>0.9272853552686484</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,62 +4280,698 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>1.973152712490546</v>
+        <v>1.701399838645164</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60</t>
+          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
+        <v>6854</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>錼創科技-KY創</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>193.0424662116648</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H73" s="2" t="n">
+        <v>37.26115285406406</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>39.63792182044081</v>
+      </c>
+      <c r="J73" s="2" t="n">
+        <v>0.504827075497997</v>
+      </c>
+      <c r="K73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N73" s="2" t="n">
+        <v>1.504382211881563</v>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>7689</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>大鵬科CLMX</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>180.6674511561264</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>28.20380236778568</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>32.172995789672</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>1.140115856278475</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>-1.182610235517359</v>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>8032</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>光菱</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>177.6478905004012</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H75" s="2" t="n">
+        <v>50.78197890962385</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>30.7338768257987</v>
+      </c>
+      <c r="J75" s="2" t="n">
+        <v>1.399501663685141</v>
+      </c>
+      <c r="K75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N75" s="2" t="n">
+        <v>0.4556695382366849</v>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>6909</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>創控</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>170.0951339405282</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>41.85</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>42.40015852246751</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>30.11710488316989</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>0.6574252603047193</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>0.3705297194905128</v>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>7703</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>銳澤</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>153.3959725847375</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H77" s="2" t="n">
+        <v>52.2358435862429</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>20.68008864281432</v>
+      </c>
+      <c r="J77" s="2" t="n">
+        <v>0.4279785520285751</v>
+      </c>
+      <c r="K77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N77" s="2" t="n">
+        <v>2.023106993773102</v>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>8038</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>長園科</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>148.7905385099617</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>32.85</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>38.79640201024616</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>20.62978018979195</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>0.4119061864070303</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>-0.0410243821268476</v>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>7770</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>君曜</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>142.2583098809928</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>39.75</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" s="2" t="n">
+        <v>52.28709347745657</v>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>12.82793555296719</v>
+      </c>
+      <c r="J79" s="2" t="n">
+        <v>0.08076032497761131</v>
+      </c>
+      <c r="K79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N79" s="2" t="n">
+        <v>0.5688200717833749</v>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>7728</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>光焱科技</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>126.305852728335</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>608</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
+        <v>47.36484555352385</v>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>17.82074134149556</v>
+      </c>
+      <c r="J80" s="2" t="n">
+        <v>0.4318038724417933</v>
+      </c>
+      <c r="K80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N80" s="2" t="n">
+        <v>5.782353699127107</v>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>ema60_gt_ema120, market_above_ma60</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>6923</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>中台</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>125.6502179615506</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>50.55926572210412</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>10.95229127344426</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.6754157054475967</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>-0.0820209368688771</v>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>7753</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>星亞</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>124.1688204529087</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>37.85</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>41.6224675178943</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>13.06905315791652</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>0.3407396361467342</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>-0.0566640056100098</v>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>6862</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>三集瑞-KY</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>114.7208036103052</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>47.30722977554326</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>22.42855587726057</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.475159423827381</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>2.959759627101038</v>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, adx_trending</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>7810</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>捷創科技</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>89.19630396848171</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>196</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
+        <v>50.99644358545656</v>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>14.912466551393</v>
+      </c>
+      <c r="J84" s="2" t="n">
+        <v>0.676627564028675</v>
+      </c>
+      <c r="K84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N84" s="2" t="n">
+        <v>1.973152712490546</v>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
         <v>6928</v>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>攸泰科技</t>
         </is>
       </c>
-      <c r="C73" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D73" s="2" t="n">
+      <c r="C85" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D85" s="2" t="n">
         <v>69.84371180756143</v>
       </c>
-      <c r="E73" s="2" t="n">
+      <c r="E85" s="2" t="n">
         <v>48.2</v>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H73" s="2" t="n">
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H85" s="2" t="n">
         <v>45.6334798691304</v>
       </c>
-      <c r="I73" s="2" t="n">
+      <c r="I85" s="2" t="n">
         <v>16.30924787513588</v>
       </c>
-      <c r="J73" s="2" t="n">
+      <c r="J85" s="2" t="n">
         <v>0.1327887778708638</v>
       </c>
-      <c r="K73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M73" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N73" s="2" t="n">
+      <c r="K85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N85" s="2" t="n">
         <v>-0.3696047203764323</v>
       </c>
-      <c r="O73" s="2" t="inlineStr">
+      <c r="O85" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>

<commit_message>
scan: seg7 2026-08-10 18:32 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-10.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-10.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>7747</v>
+        <v>7828</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>昕奇雲端</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>322.6684377577571</v>
+        <v>327.2317081791456</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>115.5</v>
+        <v>1655</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>51.55049657800621</v>
+        <v>47.77110157544003</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17.26375928080658</v>
+        <v>16.07210655007155</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1.101629169899147</v>
+        <v>0.6111243958156822</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-1.560257316981836</v>
+        <v>13.68366097496883</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>7792</v>
+        <v>7747</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>安葆</t>
+          <t>昕奇雲端</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>319.3551689189641</v>
+        <v>322.6684377577571</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>214.5</v>
+        <v>115.5</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>47.77540112805456</v>
+        <v>51.55049657800621</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>31.02575142393854</v>
+        <v>17.26375928080658</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.8361148088159112</v>
+        <v>1.101629169899147</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>3.431447458833473</v>
+        <v>-1.560257316981836</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, williams_r_recovery, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>7839</v>
+        <v>7792</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>達人網</t>
+          <t>安葆</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>307.4419975777038</v>
+        <v>319.3551689189641</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>45.5</v>
+        <v>214.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>48.27281925506811</v>
+        <v>47.77540112805456</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.48979936087653</v>
+        <v>31.02575142393854</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.7331024140356465</v>
+        <v>0.8361148088159112</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>1</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.3002111154080654</v>
+        <v>3.431447458833473</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6988</v>
+        <v>7839</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>威力暘-創</t>
+          <t>達人網</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>307.2462608016269</v>
+        <v>307.4419975777038</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>12.55</v>
+        <v>45.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>50.46653510116282</v>
+        <v>48.27281925506811</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>10.92127520834904</v>
+        <v>12.48979936087653</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1.932853922188371</v>
+        <v>0.7331024140356465</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.2361911637859376</v>
+        <v>0.3002111154080654</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>7721</v>
+        <v>6988</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>威力暘-創</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>303.7277100092821</v>
+        <v>307.2462608016269</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>62.9</v>
+        <v>12.55</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>46.96959264934583</v>
+        <v>50.46653510116282</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>25.42277511086672</v>
+        <v>10.92127520834904</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2936804443314063</v>
+        <v>1.932853922188371</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.6996548094949717</v>
+        <v>0.2361911637859376</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6865</v>
+        <v>7721</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>偉康科技</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>288.0489280430625</v>
+        <v>303.7277100092821</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>25.5</v>
+        <v>62.9</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>51.56569038885139</v>
+        <v>46.96959264934583</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>8.255619017926728</v>
+        <v>25.42277511086672</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.3895806470841059</v>
+        <v>0.2936804443314063</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.8057859384948407</v>
+        <v>0.6996548094949717</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>7705</v>
+        <v>6865</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>三商餐飲</t>
+          <t>偉康科技</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>281.0782611120818</v>
+        <v>288.0489280430625</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>31.2</v>
+        <v>25.5</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>54.48117271072788</v>
+        <v>51.56569038885139</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>19.72844289353574</v>
+        <v>8.255619017926728</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.4794116073933303</v>
+        <v>0.3895806470841059</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.141166240403041</v>
+        <v>0.8057859384948407</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6910</v>
+        <v>7705</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>德鴻</t>
+          <t>三商餐飲</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>279.5320535174742</v>
+        <v>281.0782611120818</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>25</v>
+        <v>31.2</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>45.30489816507084</v>
+        <v>54.48117271072788</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>23.82209248334926</v>
+        <v>19.72844289353574</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.909029262032193</v>
+        <v>0.4794116073933303</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.1401872102860689</v>
+        <v>0.141166240403041</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>7712</v>
+        <v>6910</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>博盛半導體</t>
+          <t>德鴻</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>279.3662481200215</v>
+        <v>279.5320535174742</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>148</v>
+        <v>25</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>49.44297980530506</v>
+        <v>45.30489816507084</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>24.40210027731012</v>
+        <v>23.82209248334926</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>1.003335673483302</v>
+        <v>0.909029262032193</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>1.999544596433511</v>
+        <v>0.1401872102860689</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>7818</v>
+        <v>7712</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>博盛半導體</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>278.8178727364322</v>
+        <v>279.3662481200215</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>63</v>
+        <v>148</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>35.60140950276744</v>
+        <v>49.44297980530506</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>34.42993761010147</v>
+        <v>24.40210027731012</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1.334145359594396</v>
+        <v>1.003335673483302</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.4636830399100147</v>
+        <v>1.999544596433511</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>7799</v>
+        <v>7818</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>266.5654036310465</v>
+        <v>278.8178727364322</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>358</v>
+        <v>63</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.96887925947232</v>
+        <v>35.60140950276744</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>20.82725411021781</v>
+        <v>34.42993761010147</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.2618675883246577</v>
+        <v>1.334145359594396</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-3.538246270219128</v>
+        <v>-0.4636830399100147</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6971</v>
+        <v>7799</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>261.7270042559304</v>
+        <v>266.5654036310465</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>25.6</v>
+        <v>358</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>33.91237872203467</v>
+        <v>42.96887925947232</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>17.01885669953462</v>
+        <v>20.82725411021781</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.8672591330968397</v>
+        <v>0.2618675883246577</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.0832816962732336</v>
+        <v>-3.538246270219128</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6994</v>
+        <v>6971</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>261.4068056261588</v>
+        <v>261.7270042559304</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>36.95</v>
+        <v>25.6</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>32.83487720384579</v>
+        <v>33.91237872203467</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>37.20335097067832</v>
+        <v>17.01885669953462</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.039352681445436</v>
+        <v>0.8672591330968397</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.2860591208910428</v>
+        <v>-0.0832816962732336</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6895</v>
+        <v>6994</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>259.0606006390066</v>
+        <v>261.4068056261588</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>118.5</v>
+        <v>36.95</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>38.55842070116779</v>
+        <v>32.83487720384579</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>26.65253592694184</v>
+        <v>37.20335097067832</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.707150545535427</v>
+        <v>1.039352681445436</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.010515000537925</v>
+        <v>0.2860591208910428</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6921</v>
+        <v>6895</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>258.3491585906293</v>
+        <v>259.0606006390066</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>65.2</v>
+        <v>118.5</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>51.70936219945977</v>
+        <v>38.55842070116779</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>27.28507203244613</v>
+        <v>26.65253592694184</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.167351073303999</v>
+        <v>0.707150545535427</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.7173881703814038</v>
+        <v>1.010515000537925</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6859</v>
+        <v>6921</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>伯特光</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>253.8726662502864</v>
+        <v>258.3491585906293</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>99.7</v>
+        <v>65.2</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>36.50236058509879</v>
+        <v>51.70936219945977</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>28.1473739515334</v>
+        <v>27.28507203244613</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.385620120895477</v>
+        <v>1.167351073303999</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.9242135344558536</v>
+        <v>0.7173881703814038</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6869</v>
+        <v>6859</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>伯特光</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>242.6743828855074</v>
+        <v>253.8726662502864</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>70.2</v>
+        <v>99.7</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>52.92645220861025</v>
+        <v>36.50236058509879</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>19.20256061100446</v>
+        <v>28.1473739515334</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>1.084395523378353</v>
+        <v>0.385620120895477</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.7016466010087159</v>
+        <v>0.9242135344558536</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>7768</v>
+        <v>6869</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>239.9041356068924</v>
+        <v>242.6743828855074</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>261.5</v>
+        <v>70.2</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>35.83878580896345</v>
+        <v>52.92645220861025</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>45.16833733265</v>
+        <v>19.20256061100446</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4331677512119838</v>
+        <v>1.084395523378353</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>1.886270425394073</v>
+        <v>0.7016466010087159</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6908</v>
+        <v>7768</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>239.5553009001952</v>
+        <v>239.9041356068924</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>32.9</v>
+        <v>261.5</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.12329248450961</v>
+        <v>35.83878580896345</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>31.5423807528287</v>
+        <v>45.16833733265</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1.02796052631579</v>
+        <v>0.4331677512119838</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.07725547166748289</v>
+        <v>1.886270425394073</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6887</v>
+        <v>6908</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>236.8265361674669</v>
+        <v>239.5553009001952</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>36.05</v>
+        <v>32.9</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>47.83771172224126</v>
+        <v>36.12329248450961</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.00962407669346</v>
+        <v>31.5423807528287</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.2060087555679954</v>
+        <v>1.02796052631579</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.185212618965927</v>
+        <v>-0.07725547166748289</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6906</v>
+        <v>6887</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>233.0092844365423</v>
+        <v>236.8265361674669</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>71</v>
+        <v>36.05</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>40.56464498373511</v>
+        <v>47.83771172224126</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>29.34192093776815</v>
+        <v>17.00962407669346</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.9136662795199382</v>
+        <v>0.2060087555679954</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.7920186934425986</v>
+        <v>-0.185212618965927</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>7749</v>
+        <v>6906</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>230.2345308208552</v>
+        <v>233.0092844365423</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>355.5</v>
+        <v>71</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>44.64577207325237</v>
+        <v>40.56464498373511</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>32.27720967521438</v>
+        <v>29.34192093776815</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6268777173692717</v>
+        <v>0.9136662795199382</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>5.34143688898196</v>
+        <v>0.7920186934425986</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6899</v>
+        <v>7749</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>224.3041518260263</v>
+        <v>230.2345308208552</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>50.7</v>
+        <v>355.5</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>38.06729527396745</v>
+        <v>44.64577207325237</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>23.54492871355304</v>
+        <v>32.27720967521438</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4908126190059958</v>
+        <v>0.6268777173692717</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.3486261016285426</v>
+        <v>5.34143688898196</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6953</v>
+        <v>6899</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>220.6802644635352</v>
+        <v>224.3041518260263</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>223</v>
+        <v>50.7</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,16 +5375,16 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>52.95213263675682</v>
+        <v>38.06729527396745</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>9.894791767196232</v>
+        <v>23.54492871355304</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.3082033120190888</v>
+        <v>0.4908126190059958</v>
       </c>
       <c r="K93" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>1.788417789291647</v>
+        <v>0.3486261016285426</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend, dealer_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>7823</v>
+        <v>6953</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>220.2788723864819</v>
+        <v>220.6802644635352</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>83.7</v>
+        <v>223</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>52.32761355074214</v>
+        <v>52.95213263675682</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>18.01839511503825</v>
+        <v>9.894791767196232</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1.645009747760591</v>
+        <v>0.3082033120190888</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.6048660408889529</v>
+        <v>1.788417789291647</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, stronger_than_market</t>
+          <t>market_above_ma60, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6873</v>
+        <v>7823</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>215.0974662222889</v>
+        <v>220.2788723864819</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>79</v>
+        <v>83.7</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>43.20207975417044</v>
+        <v>52.32761355074214</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.63486014762306</v>
+        <v>18.01839511503825</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1.10646005076004</v>
+        <v>1.645009747760591</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.3468792592392931</v>
+        <v>0.6048660408889529</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>8034</v>
+        <v>6873</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>214.1047081881592</v>
+        <v>215.0974662222889</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>19.1</v>
+        <v>79</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>39.79083766211048</v>
+        <v>43.20207975417044</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>36.10566422157577</v>
+        <v>16.63486014762306</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6850546000333173</v>
+        <v>1.10646005076004</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.1409505553634835</v>
+        <v>-0.3468792592392931</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6965</v>
+        <v>8034</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>211.9851754548217</v>
+        <v>214.1047081881592</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>77</v>
+        <v>19.1</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>44.74043742353538</v>
+        <v>39.79083766211048</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>31.69511478903778</v>
+        <v>36.10566422157577</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3032927773685304</v>
+        <v>0.6850546000333173</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.0881056404112585</v>
+        <v>0.1409505553634835</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5615,21 +5615,21 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6894</v>
+        <v>6965</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>209.6960034481655</v>
+        <v>211.9851754548217</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>346.5</v>
+        <v>77</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>53.05600793743652</v>
+        <v>44.74043742353538</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>16.31462079186515</v>
+        <v>31.69511478903778</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.7580949872617595</v>
+        <v>0.3032927773685304</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>4.406072900351855</v>
+        <v>-0.0881056404112585</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8024</v>
+        <v>6894</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>209.6240690164325</v>
+        <v>209.6960034481655</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>14.1</v>
+        <v>346.5</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.03815138841021</v>
+        <v>53.05600793743652</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>18.49613831537289</v>
+        <v>16.31462079186515</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.6706454070423011</v>
+        <v>0.7580949872617595</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.1398571671965818</v>
+        <v>4.406072900351855</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5721,21 +5721,21 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6877</v>
+        <v>8024</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>209.4432275446592</v>
+        <v>209.6240690164325</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>127.5</v>
+        <v>14.1</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>52.24148104051165</v>
+        <v>44.03815138841021</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.53708461897214</v>
+        <v>18.49613831537289</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.8661062567621975</v>
+        <v>0.6706454070423011</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>1.500200763685784</v>
+        <v>-0.1398571671965818</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>7402</v>
+        <v>6877</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>207.5863099348092</v>
+        <v>209.4432275446592</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>103</v>
+        <v>127.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.19251715783129</v>
+        <v>52.24148104051165</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>20.63468970003154</v>
+        <v>18.53708461897214</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.149618364569397</v>
+        <v>0.8661062567621975</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>1</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.7599105654133251</v>
+        <v>1.500200763685784</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7842</v>
+        <v>7402</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>204.0135455639476</v>
+        <v>207.5863099348092</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>91.59999999999999</v>
+        <v>103</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>53.00345780940963</v>
+        <v>44.19251715783129</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>10.26079279614132</v>
+        <v>20.63468970003154</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1.6562574970012</v>
+        <v>0.149618364569397</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>1.205609064200336</v>
+        <v>-0.7599105654133251</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6925</v>
+        <v>7842</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>201.4719139133944</v>
+        <v>204.0135455639476</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>54.4</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>46.75529556895629</v>
+        <v>53.00345780940963</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.42012752347143</v>
+        <v>10.26079279614132</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.6822738615546613</v>
+        <v>1.6562574970012</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.4604532178979621</v>
+        <v>1.205609064200336</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, stronger_than_market</t>
+          <t>volume_break, market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6967</v>
+        <v>6925</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>196.6235767539877</v>
+        <v>201.4719139133944</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>69.3</v>
+        <v>54.4</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>45.52480241209469</v>
+        <v>46.75529556895629</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>16.49585506093718</v>
+        <v>16.42012752347143</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.08774113964356781</v>
+        <v>0.6822738615546613</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.3162031130703682</v>
+        <v>0.4604532178979621</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>7791</v>
+        <v>6967</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>195.7222183759985</v>
+        <v>196.6235767539877</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>59.7</v>
+        <v>69.3</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>33.31213615253978</v>
+        <v>45.52480241209469</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>25.1816493173711</v>
+        <v>16.49585506093718</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.4388103277519661</v>
+        <v>0.08774113964356781</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1138288335024849</v>
+        <v>-0.3162031130703682</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6924</v>
+        <v>7791</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>193.2275993596958</v>
+        <v>195.7222183759985</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>109</v>
+        <v>59.7</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>47.51677580480385</v>
+        <v>33.31213615253978</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.47828919063415</v>
+        <v>25.1816493173711</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.9272853552686484</v>
+        <v>0.4388103277519661</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>1.701399838645164</v>
+        <v>-0.1138288335024849</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6854</v>
+        <v>6924</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>193.0424662116648</v>
+        <v>193.2275993596958</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>94.2</v>
+        <v>109</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>37.26115285406406</v>
+        <v>47.51677580480385</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>39.63792182044081</v>
+        <v>18.47828919063415</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.504827075497997</v>
+        <v>0.9272853552686484</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>1.504382211881563</v>
+        <v>1.701399838645164</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>7689</v>
+        <v>6854</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>180.6674511561264</v>
+        <v>193.0424662116648</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>171.5</v>
+        <v>94.2</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>28.20380236778568</v>
+        <v>37.26115285406406</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>32.172995789672</v>
+        <v>39.63792182044081</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1.140115856278475</v>
+        <v>0.504827075497997</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-1.182610235517359</v>
+        <v>1.504382211881563</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>7803</v>
+        <v>7689</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>179.1084174680117</v>
+        <v>180.6674511561264</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>19.7</v>
+        <v>171.5</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>38.60155730137843</v>
+        <v>28.20380236778568</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>21.58682327471746</v>
+        <v>32.172995789672</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.4704432163680859</v>
+        <v>1.140115856278475</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0462741349279085</v>
+        <v>-1.182610235517359</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6251,21 +6251,21 @@
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8032</v>
+        <v>7803</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>177.6478905004012</v>
+        <v>179.1084174680117</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>37.9</v>
+        <v>19.7</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>50.78197890962385</v>
+        <v>38.60155730137843</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>30.7338768257987</v>
+        <v>21.58682327471746</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.399501663685141</v>
+        <v>0.4704432163680859</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.4556695382366849</v>
+        <v>0.0462741349279085</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6885</v>
+        <v>8032</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>174.913882640098</v>
+        <v>177.6478905004012</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>20.55</v>
+        <v>37.9</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.19456218353822</v>
+        <v>50.78197890962385</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.02345253649756</v>
+        <v>30.7338768257987</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>1.051167406610397</v>
+        <v>1.399501663685141</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0471231515670762</v>
+        <v>0.4556695382366849</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6909</v>
+        <v>6885</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>170.0951339405282</v>
+        <v>174.913882640098</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>41.85</v>
+        <v>20.55</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>42.40015852246751</v>
+        <v>42.19456218353822</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>30.11710488316989</v>
+        <v>11.02345253649756</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.6574252603047193</v>
+        <v>1.051167406610397</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.3705297194905128</v>
+        <v>0.0471231515670762</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6997</v>
+        <v>6909</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>166.6946000277282</v>
+        <v>170.0951339405282</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0</v>
+        <v>41.85</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>40.603896681415</v>
+        <v>42.40015852246751</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>11.85472681196761</v>
+        <v>30.11710488316989</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.0182285375441987</v>
+        <v>0.6574252603047193</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1017937378236508</v>
+        <v>0.3705297194905128</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>7703</v>
+        <v>6997</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>銳澤</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>153.3959725847375</v>
+        <v>166.6946000277282</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>185</v>
+        <v>0</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>52.2358435862429</v>
+        <v>40.603896681415</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>20.68008864281432</v>
+        <v>11.85472681196761</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.4279785520285751</v>
+        <v>0.0182285375441987</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>2.023106993773102</v>
+        <v>-0.1017937378236508</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>8038</v>
+        <v>7703</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>銳澤</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>148.7905385099617</v>
+        <v>153.3959725847375</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>32.85</v>
+        <v>185</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>38.79640201024616</v>
+        <v>52.2358435862429</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>20.62978018979195</v>
+        <v>20.68008864281432</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.4119061864070303</v>
+        <v>0.4279785520285751</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0410243821268476</v>
+        <v>2.023106993773102</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6934</v>
+        <v>8038</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>143.4279535584905</v>
+        <v>148.7905385099617</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>72</v>
+        <v>32.85</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.05189006533956</v>
+        <v>38.79640201024616</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>17.17712536058581</v>
+        <v>20.62978018979195</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6601581160639193</v>
+        <v>0.4119061864070303</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.8137889692630491</v>
+        <v>-0.0410243821268476</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>7770</v>
+        <v>6934</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>142.2583098809928</v>
+        <v>143.4279535584905</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>39.75</v>
+        <v>72</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>52.28709347745657</v>
+        <v>43.05189006533956</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.82793555296719</v>
+        <v>17.17712536058581</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.08076032497761131</v>
+        <v>0.6601581160639193</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.5688200717833749</v>
+        <v>-0.8137889692630491</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7765</v>
+        <v>7770</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>129.9938563418593</v>
+        <v>142.2583098809928</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>225.5</v>
+        <v>39.75</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>49.26095069634169</v>
+        <v>52.28709347745657</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>12.49443651617659</v>
+        <v>12.82793555296719</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.5982814368522649</v>
+        <v>0.08076032497761131</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.5184406365553724</v>
+        <v>0.5688200717833749</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>7728</v>
+        <v>7765</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>126.305852728335</v>
+        <v>129.9938563418593</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>608</v>
+        <v>225.5</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>47.36484555352385</v>
+        <v>49.26095069634169</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.82074134149556</v>
+        <v>12.49443651617659</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4318038724417933</v>
+        <v>0.5982814368522649</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>5.782353699127107</v>
+        <v>0.5184406365553724</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6923</v>
+        <v>7728</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>125.6502179615506</v>
+        <v>126.305852728335</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>76.7</v>
+        <v>608</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>50.55926572210412</v>
+        <v>47.36484555352385</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>10.95229127344426</v>
+        <v>17.82074134149556</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.6754157054475967</v>
+        <v>0.4318038724417933</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0820209368688771</v>
+        <v>5.782353699127107</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7753</v>
+        <v>6923</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>124.1688204529087</v>
+        <v>125.6502179615506</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>37.85</v>
+        <v>76.7</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.6224675178943</v>
+        <v>50.55926572210412</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>13.06905315791652</v>
+        <v>10.95229127344426</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.3407396361467342</v>
+        <v>0.6754157054475967</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.0566640056100098</v>
+        <v>-0.0820209368688771</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6862</v>
+        <v>7753</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>114.7208036103052</v>
+        <v>124.1688204529087</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>149</v>
+        <v>37.85</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>47.30722977554326</v>
+        <v>41.6224675178943</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>22.42855587726057</v>
+        <v>13.06905315791652</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.475159423827381</v>
+        <v>0.3407396361467342</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>2.959759627101038</v>
+        <v>-0.0566640056100098</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>7760</v>
+        <v>6862</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>106.9829545217051</v>
+        <v>114.7208036103052</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>33.15</v>
+        <v>149</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>41.52897759544516</v>
+        <v>47.30722977554326</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>14.77333277022284</v>
+        <v>22.42855587726057</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.2860025731529375</v>
+        <v>0.475159423827381</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.1697933851964378</v>
+        <v>2.959759627101038</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>7810</v>
+        <v>7760</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>89.19630396848171</v>
+        <v>106.9829545217051</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>196</v>
+        <v>33.15</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>50.99644358545656</v>
+        <v>41.52897759544516</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>14.912466551393</v>
+        <v>14.77333277022284</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.676627564028675</v>
+        <v>0.2860025731529375</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>1.973152712490546</v>
+        <v>-0.1697933851964378</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6928</v>
+        <v>7810</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>捷創科技</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>69.84371180756143</v>
+        <v>89.19630396848171</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>48.2</v>
+        <v>196</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>45.6334798691304</v>
+        <v>50.99644358545656</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.30924787513588</v>
+        <v>14.912466551393</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.1327887778708638</v>
+        <v>0.676627564028675</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,62 +7089,115 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.3696047203764323</v>
+        <v>1.973152712490546</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
+        <v>6928</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>攸泰科技</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>69.84371180756143</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>45.6334798691304</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>16.30924787513588</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.1327887778708638</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>-0.3696047203764323</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>7736</v>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>虎山</t>
         </is>
       </c>
-      <c r="C126" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D126" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>58.37072666185427</v>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>44.05597019909899</v>
       </c>
-      <c r="I126" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>18.20494115559537</v>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.3742122362704035</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N126" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>0.0296943513908846</v>
       </c>
-      <c r="O126" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>